<commit_message>
generated tables for all cost factors up to 100. organised into folders
</commit_message>
<xml_diff>
--- a/plots/higher_costs/N_16/constructing_table/analysis/building_table_results.xlsx
+++ b/plots/higher_costs/N_16/constructing_table/analysis/building_table_results.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\psymf9\PhD Repositories\cherry-picking-reduction-functions\plots\higher_costs\N_16\constructing_table\analysis\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{2DA47704-B1F6-4515-A2DF-7B338D011281}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{8DDEC19D-1D8E-4489-B768-20F7D4E9BCA9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1950" yWindow="1950" windowWidth="21600" windowHeight="11295" xr2:uid="{3F557E5A-1160-48D2-9D43-BF41C9EB42CC}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{3F557E5A-1160-48D2-9D43-BF41C9EB42CC}"/>
   </bookViews>
   <sheets>
     <sheet name="building_table_results" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="17">
   <si>
     <t>cost_factor</t>
   </si>
@@ -41,6 +41,36 @@
   </si>
   <si>
     <t>duration</t>
+  </si>
+  <si>
+    <t>Cost</t>
+  </si>
+  <si>
+    <t>Costs</t>
+  </si>
+  <si>
+    <t>Reduce</t>
+  </si>
+  <si>
+    <t>Hash</t>
+  </si>
+  <si>
+    <t>Actual Cost</t>
+  </si>
+  <si>
+    <t>m_t</t>
+  </si>
+  <si>
+    <t>Cost Factor</t>
+  </si>
+  <si>
+    <t>Duration</t>
+  </si>
+  <si>
+    <t>Vanilla</t>
+  </si>
+  <si>
+    <t>vanilla</t>
   </si>
 </sst>
 </file>
@@ -183,7 +213,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="33">
+  <fills count="36">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -363,8 +393,26 @@
         <bgColor indexed="65"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF00B0F0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF92D050"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC000"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="10">
+  <borders count="21">
     <border>
       <left/>
       <right/>
@@ -477,6 +525,133 @@
       <bottom style="double">
         <color theme="4"/>
       </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
       <diagonal/>
     </border>
   </borders>
@@ -524,8 +699,78 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="33">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="33" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="34" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="34" borderId="10" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="33" borderId="16" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="34" borderId="17" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="33" borderId="11" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="34" borderId="12" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="34" borderId="18" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="34" borderId="19" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="33" borderId="18" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="33" borderId="19" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="10" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -901,33 +1146,46 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{52475418-B3BB-434B-8C92-20FCA0178835}">
-  <dimension ref="A1:G7"/>
+  <dimension ref="A1:O42"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="13.7109375" customWidth="1"/>
+    <col min="2" max="2" width="18.28515625" customWidth="1"/>
+    <col min="3" max="3" width="16.5703125" customWidth="1"/>
+    <col min="4" max="4" width="17.140625" customWidth="1"/>
+    <col min="5" max="5" width="12.140625" customWidth="1"/>
+    <col min="6" max="7" width="16" customWidth="1"/>
+    <col min="8" max="8" width="17" customWidth="1"/>
+    <col min="15" max="15" width="10.28515625" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
+    <row r="1" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="H1" s="1" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>5</v>
       </c>
@@ -947,10 +1205,18 @@
         <v>863541440</v>
       </c>
       <c r="G2">
+        <f>E2+(F2*O3)</f>
+        <v>4150309.1333213709</v>
+      </c>
+      <c r="H2">
         <v>330.16673819999698</v>
       </c>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="N2" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="O2" s="2"/>
+    </row>
+    <row r="3" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>10</v>
       </c>
@@ -970,10 +1236,21 @@
         <v>1975300366</v>
       </c>
       <c r="G3">
+        <f>E3+(F3*O3)</f>
+        <v>6145211.2076081112</v>
+      </c>
+      <c r="H3">
         <v>761.58847739999999</v>
       </c>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="N3" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="O3">
+        <f xml:space="preserve"> 1/557.3</f>
+        <v>1.7943656917279744E-3</v>
+      </c>
+    </row>
+    <row r="4" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>15</v>
       </c>
@@ -993,10 +1270,20 @@
         <v>3078534119</v>
       </c>
       <c r="G4">
+        <f>E4+(F4*O3)</f>
+        <v>8124816.0039476054</v>
+      </c>
+      <c r="H4">
         <v>1224.3331814000001</v>
       </c>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="N4" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="O4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>20</v>
       </c>
@@ -1016,10 +1303,14 @@
         <v>4189736966</v>
       </c>
       <c r="G5">
+        <f>E5+(F5*O3)</f>
+        <v>10118720.269154854</v>
+      </c>
+      <c r="H5">
         <v>1659.8530086999999</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>25</v>
       </c>
@@ -1039,10 +1330,14 @@
         <v>5288083229</v>
       </c>
       <c r="G6">
+        <f>E6+(F6*O3)</f>
+        <v>12089555.121119685</v>
+      </c>
+      <c r="H6">
         <v>2044.2409072999999</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>30</v>
       </c>
@@ -1062,10 +1357,573 @@
         <v>6403915448</v>
       </c>
       <c r="G7">
+        <f>E7+(F7*O3)</f>
+        <v>14091766.172617981</v>
+      </c>
+      <c r="H7">
         <v>2454.4015013999901</v>
       </c>
     </row>
+    <row r="12" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="B12" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="C12" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="D12" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="E12" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="F12" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="G12" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="H12" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="I12" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="13" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="B13">
+        <v>5</v>
+      </c>
+      <c r="C13" s="3">
+        <v>2270</v>
+      </c>
+      <c r="D13" s="6">
+        <v>2197</v>
+      </c>
+      <c r="E13" s="3">
+        <v>2026772.68405492</v>
+      </c>
+      <c r="F13">
+        <v>2600800</v>
+      </c>
+      <c r="G13">
+        <v>863541440</v>
+      </c>
+      <c r="H13" s="6">
+        <v>4150309.1333213709</v>
+      </c>
+      <c r="I13">
+        <v>330.16673819999698</v>
+      </c>
+    </row>
+    <row r="14" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="B14">
+        <v>10</v>
+      </c>
+      <c r="C14" s="3">
+        <v>2317</v>
+      </c>
+      <c r="D14" s="6">
+        <v>2245</v>
+      </c>
+      <c r="E14" s="3">
+        <v>4053545.3778719199</v>
+      </c>
+      <c r="F14">
+        <v>2600800</v>
+      </c>
+      <c r="G14">
+        <v>1975300366</v>
+      </c>
+      <c r="H14" s="6">
+        <v>6145211.2076081112</v>
+      </c>
+      <c r="I14">
+        <v>761.58847739999999</v>
+      </c>
+    </row>
+    <row r="15" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="B15">
+        <v>15</v>
+      </c>
+      <c r="C15" s="3">
+        <v>2341</v>
+      </c>
+      <c r="D15" s="6">
+        <v>2264</v>
+      </c>
+      <c r="E15" s="3">
+        <v>6080318.0443998799</v>
+      </c>
+      <c r="F15">
+        <v>2600800</v>
+      </c>
+      <c r="G15">
+        <v>3078534119</v>
+      </c>
+      <c r="H15" s="6">
+        <v>8124816.0039476054</v>
+      </c>
+      <c r="I15">
+        <v>1224.3331814000001</v>
+      </c>
+    </row>
+    <row r="16" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="B16">
+        <v>20</v>
+      </c>
+      <c r="C16" s="3">
+        <v>2358</v>
+      </c>
+      <c r="D16" s="6">
+        <v>2277</v>
+      </c>
+      <c r="E16" s="3">
+        <v>8107090.7553425403</v>
+      </c>
+      <c r="F16">
+        <v>2600800</v>
+      </c>
+      <c r="G16">
+        <v>4189736966</v>
+      </c>
+      <c r="H16" s="6">
+        <v>10118720.269154854</v>
+      </c>
+      <c r="I16">
+        <v>1659.8530086999999</v>
+      </c>
+    </row>
+    <row r="17" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B17">
+        <v>25</v>
+      </c>
+      <c r="C17" s="3">
+        <v>2371</v>
+      </c>
+      <c r="D17" s="6">
+        <v>2276</v>
+      </c>
+      <c r="E17" s="3">
+        <v>10133863.377056301</v>
+      </c>
+      <c r="F17">
+        <v>2600800</v>
+      </c>
+      <c r="G17">
+        <v>5288083229</v>
+      </c>
+      <c r="H17" s="6">
+        <v>12089555.121119685</v>
+      </c>
+      <c r="I17">
+        <v>2044.2409072999999</v>
+      </c>
+    </row>
+    <row r="18" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B18">
+        <v>30</v>
+      </c>
+      <c r="C18" s="3">
+        <v>2381</v>
+      </c>
+      <c r="D18" s="6">
+        <v>2291</v>
+      </c>
+      <c r="E18" s="3">
+        <v>12160635.9783941</v>
+      </c>
+      <c r="F18">
+        <v>2600800</v>
+      </c>
+      <c r="G18">
+        <v>6403915448</v>
+      </c>
+      <c r="H18" s="6">
+        <v>14091766.172617981</v>
+      </c>
+      <c r="I18">
+        <v>2454.4015013999901</v>
+      </c>
+    </row>
+    <row r="22" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B22" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="C22" s="12" t="s">
+        <v>12</v>
+      </c>
+      <c r="D22" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="E22" s="4" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="23" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B23" s="19" t="s">
+        <v>15</v>
+      </c>
+      <c r="C23" s="20">
+        <v>1563</v>
+      </c>
+      <c r="D23" s="21">
+        <v>2600800</v>
+      </c>
+      <c r="E23" s="21">
+        <v>4.1357776000077102</v>
+      </c>
+    </row>
+    <row r="24" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B24" s="8">
+        <v>5</v>
+      </c>
+      <c r="C24" s="10">
+        <v>2270</v>
+      </c>
+      <c r="D24" s="13">
+        <v>2026772.68405492</v>
+      </c>
+      <c r="E24" s="15">
+        <v>330.16673819999698</v>
+      </c>
+    </row>
+    <row r="25" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B25" s="8"/>
+      <c r="C25" s="11">
+        <v>2197</v>
+      </c>
+      <c r="D25" s="14">
+        <v>4150309.1333213709</v>
+      </c>
+      <c r="E25" s="16"/>
+    </row>
+    <row r="26" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B26" s="22"/>
+      <c r="C26" s="23"/>
+      <c r="D26" s="24"/>
+      <c r="E26" s="25"/>
+    </row>
+    <row r="27" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B27" s="8">
+        <v>10</v>
+      </c>
+      <c r="C27" s="10">
+        <v>2317</v>
+      </c>
+      <c r="D27" s="13">
+        <v>4053545.3778719199</v>
+      </c>
+      <c r="E27" s="15">
+        <v>761.58847739999999</v>
+      </c>
+      <c r="G27" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="H27" s="31">
+        <v>0.85409999999999997</v>
+      </c>
+      <c r="I27" s="5">
+        <v>1726.91</v>
+      </c>
+      <c r="J27" s="7">
+        <v>11.45</v>
+      </c>
+    </row>
+    <row r="28" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B28" s="8"/>
+      <c r="C28" s="26"/>
+      <c r="D28" s="27"/>
+      <c r="E28" s="28"/>
+      <c r="G28" s="5"/>
+      <c r="H28" s="31"/>
+      <c r="I28" s="5"/>
+      <c r="J28" s="32">
+        <v>52.46</v>
+      </c>
+    </row>
+    <row r="29" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B29" s="8"/>
+      <c r="C29" s="11">
+        <v>2245</v>
+      </c>
+      <c r="D29" s="14">
+        <v>6145211.2076081112</v>
+      </c>
+      <c r="E29" s="16"/>
+      <c r="G29" s="5">
+        <v>5</v>
+      </c>
+      <c r="H29" s="31">
+        <v>0.93259999999999998</v>
+      </c>
+      <c r="I29" s="5">
+        <v>1347.63</v>
+      </c>
+      <c r="J29" s="7">
+        <v>10.87</v>
+      </c>
+    </row>
+    <row r="30" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B30" s="22"/>
+      <c r="C30" s="23"/>
+      <c r="D30" s="24"/>
+      <c r="E30" s="25"/>
+      <c r="G30" s="5"/>
+      <c r="H30" s="31"/>
+      <c r="I30" s="5"/>
+      <c r="J30" s="32">
+        <v>57.91</v>
+      </c>
+    </row>
+    <row r="31" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B31" s="8">
+        <v>15</v>
+      </c>
+      <c r="C31" s="10">
+        <v>2341</v>
+      </c>
+      <c r="D31" s="13">
+        <v>6080318.0443998799</v>
+      </c>
+      <c r="E31" s="15">
+        <v>1224.3331814000001</v>
+      </c>
+      <c r="G31" s="5">
+        <v>10</v>
+      </c>
+      <c r="H31" s="31">
+        <v>0.9385</v>
+      </c>
+      <c r="I31" s="5">
+        <v>1304.79</v>
+      </c>
+      <c r="J31" s="7">
+        <v>10.63</v>
+      </c>
+    </row>
+    <row r="32" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B32" s="8"/>
+      <c r="C32" s="26"/>
+      <c r="D32" s="27"/>
+      <c r="E32" s="28"/>
+      <c r="G32" s="5"/>
+      <c r="H32" s="31"/>
+      <c r="I32" s="5"/>
+      <c r="J32" s="32">
+        <v>57.89</v>
+      </c>
+    </row>
+    <row r="33" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B33" s="8"/>
+      <c r="C33" s="11">
+        <v>2264</v>
+      </c>
+      <c r="D33" s="14">
+        <v>8124816.0039476054</v>
+      </c>
+      <c r="E33" s="16"/>
+      <c r="G33" s="5">
+        <v>15</v>
+      </c>
+      <c r="H33" s="31">
+        <v>0.93930000000000002</v>
+      </c>
+      <c r="I33" s="5">
+        <v>1294.01</v>
+      </c>
+      <c r="J33" s="7">
+        <v>10.54</v>
+      </c>
+    </row>
+    <row r="34" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B34" s="22"/>
+      <c r="C34" s="23"/>
+      <c r="D34" s="24"/>
+      <c r="E34" s="29"/>
+      <c r="G34" s="5"/>
+      <c r="H34" s="31"/>
+      <c r="I34" s="5"/>
+      <c r="J34" s="32">
+        <v>57.88</v>
+      </c>
+    </row>
+    <row r="35" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B35" s="8">
+        <v>20</v>
+      </c>
+      <c r="C35" s="10">
+        <v>2358</v>
+      </c>
+      <c r="D35" s="13">
+        <v>8107090.7553425403</v>
+      </c>
+      <c r="E35" s="17">
+        <v>1659.8530086999999</v>
+      </c>
+      <c r="G35" s="5">
+        <v>20</v>
+      </c>
+      <c r="H35" s="31">
+        <v>0.94140000000000001</v>
+      </c>
+      <c r="I35" s="5">
+        <v>1291.77</v>
+      </c>
+      <c r="J35" s="7">
+        <v>10.65</v>
+      </c>
+    </row>
+    <row r="36" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B36" s="8"/>
+      <c r="C36" s="26"/>
+      <c r="D36" s="27"/>
+      <c r="E36" s="30"/>
+      <c r="G36" s="5"/>
+      <c r="H36" s="31"/>
+      <c r="I36" s="5"/>
+      <c r="J36" s="32">
+        <v>58.27</v>
+      </c>
+    </row>
+    <row r="37" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B37" s="8"/>
+      <c r="C37" s="11">
+        <v>2277</v>
+      </c>
+      <c r="D37" s="14">
+        <v>10118720.269154854</v>
+      </c>
+      <c r="E37" s="18"/>
+      <c r="G37" s="5">
+        <v>25</v>
+      </c>
+      <c r="H37" s="31">
+        <v>0.94089999999999996</v>
+      </c>
+      <c r="I37" s="5">
+        <v>1290.5</v>
+      </c>
+      <c r="J37" s="7">
+        <v>10.6</v>
+      </c>
+    </row>
+    <row r="38" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B38" s="22"/>
+      <c r="C38" s="23"/>
+      <c r="D38" s="24"/>
+      <c r="E38" s="29"/>
+      <c r="G38" s="5"/>
+      <c r="H38" s="31"/>
+      <c r="I38" s="5"/>
+      <c r="J38" s="32">
+        <v>58.06</v>
+      </c>
+    </row>
+    <row r="39" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B39" s="8">
+        <v>25</v>
+      </c>
+      <c r="C39" s="10">
+        <v>2371</v>
+      </c>
+      <c r="D39" s="13">
+        <v>10133863.377056301</v>
+      </c>
+      <c r="E39" s="17">
+        <v>2044.2409072999999</v>
+      </c>
+      <c r="G39" s="5">
+        <v>30</v>
+      </c>
+      <c r="H39" s="31">
+        <v>0.94089999999999996</v>
+      </c>
+      <c r="I39" s="5">
+        <v>1296.31</v>
+      </c>
+      <c r="J39" s="7">
+        <v>10.7</v>
+      </c>
+    </row>
+    <row r="40" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B40" s="8"/>
+      <c r="C40" s="11">
+        <v>2276</v>
+      </c>
+      <c r="D40" s="14">
+        <v>12089555.121119685</v>
+      </c>
+      <c r="E40" s="18"/>
+      <c r="G40" s="5"/>
+      <c r="H40" s="31"/>
+      <c r="I40" s="5"/>
+      <c r="J40" s="32">
+        <v>58.45</v>
+      </c>
+    </row>
+    <row r="41" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B41" s="8">
+        <v>30</v>
+      </c>
+      <c r="C41" s="10">
+        <v>2381</v>
+      </c>
+      <c r="D41" s="13">
+        <v>12160635.9783941</v>
+      </c>
+      <c r="E41" s="17">
+        <v>2454.4015013999901</v>
+      </c>
+    </row>
+    <row r="42" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B42" s="8"/>
+      <c r="C42" s="11">
+        <v>2291</v>
+      </c>
+      <c r="D42" s="14">
+        <v>14091766.172617981</v>
+      </c>
+      <c r="E42" s="18"/>
+    </row>
   </sheetData>
+  <mergeCells count="34">
+    <mergeCell ref="H37:H38"/>
+    <mergeCell ref="I27:I28"/>
+    <mergeCell ref="I29:I30"/>
+    <mergeCell ref="I31:I32"/>
+    <mergeCell ref="I33:I34"/>
+    <mergeCell ref="I35:I36"/>
+    <mergeCell ref="I37:I38"/>
+    <mergeCell ref="G35:G36"/>
+    <mergeCell ref="G33:G34"/>
+    <mergeCell ref="G31:G32"/>
+    <mergeCell ref="G29:G30"/>
+    <mergeCell ref="G27:G28"/>
+    <mergeCell ref="H27:H28"/>
+    <mergeCell ref="H29:H30"/>
+    <mergeCell ref="H31:H32"/>
+    <mergeCell ref="H33:H34"/>
+    <mergeCell ref="H35:H36"/>
+    <mergeCell ref="B41:B42"/>
+    <mergeCell ref="E24:E25"/>
+    <mergeCell ref="E27:E29"/>
+    <mergeCell ref="E31:E33"/>
+    <mergeCell ref="E35:E37"/>
+    <mergeCell ref="E39:E40"/>
+    <mergeCell ref="E41:E42"/>
+    <mergeCell ref="N2:O2"/>
+    <mergeCell ref="B24:B25"/>
+    <mergeCell ref="B27:B29"/>
+    <mergeCell ref="B31:B33"/>
+    <mergeCell ref="B35:B37"/>
+    <mergeCell ref="B39:B40"/>
+    <mergeCell ref="I39:I40"/>
+    <mergeCell ref="H39:H40"/>
+    <mergeCell ref="G39:G40"/>
+    <mergeCell ref="G37:G38"/>
+  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>